<commit_message>
elimina estudiantes sin respuestas (SHARON RAMIREZ GIRALDA 501, LESLY VILLALBA BUENAVISTA 1101)
</commit_message>
<xml_diff>
--- a/PRUEBAS A CALIFICAR/Ya procesadas/COLEGIO-BUENAVISTA-(IED)-1101_20260625_104109.xlsx
+++ b/PRUEBAS A CALIFICAR/Ya procesadas/COLEGIO-BUENAVISTA-(IED)-1101_20260625_104109.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Catherine Espinosa\Desktop\ORIGINALES PRUEBAS\18-06-2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Catherine Espinosa\Desktop\PROYECTO JULIANA\PRUEBAS A CALIFICAR\Ya procesadas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25DA7BBE-2B89-48CF-B383-81D63C3114F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0342D793-6EB0-473A-B6C6-0F1BD12A630B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,14 +16,14 @@
     <sheet name="Resultados" sheetId="4" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Resultados!$A$1:$AB$65</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Resultados!$A$1:$AB$63</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1648" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1636" uniqueCount="99">
   <si>
     <t>Pág</t>
   </si>
@@ -317,12 +317,6 @@
   </si>
   <si>
     <t>1028868450</t>
-  </si>
-  <si>
-    <t>LESLY SOFIA VILLALBA SANCHEZ</t>
-  </si>
-  <si>
-    <t>1029280271</t>
   </si>
   <si>
     <t>matematicas</t>
@@ -707,7 +701,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADB2070B-47CF-4426-A87A-6271E231ACA6}">
-  <dimension ref="A1:AB65"/>
+  <dimension ref="A1:AB63"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="11.81640625" bestFit="1" customWidth="1"/>
@@ -2693,7 +2687,7 @@
     </row>
     <row r="24" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A24">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B24">
         <v>111001100013</v>
@@ -2702,10 +2696,10 @@
         <v>28</v>
       </c>
       <c r="D24" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="E24" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="F24" t="s">
         <v>31</v>
@@ -2716,10 +2710,70 @@
       <c r="H24" t="s">
         <v>33</v>
       </c>
+      <c r="I24" t="s">
+        <v>37</v>
+      </c>
+      <c r="J24" t="s">
+        <v>34</v>
+      </c>
+      <c r="K24" t="s">
+        <v>34</v>
+      </c>
+      <c r="L24" t="s">
+        <v>37</v>
+      </c>
+      <c r="M24" t="s">
+        <v>35</v>
+      </c>
+      <c r="N24" t="s">
+        <v>37</v>
+      </c>
+      <c r="O24" t="s">
+        <v>34</v>
+      </c>
+      <c r="P24" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>37</v>
+      </c>
+      <c r="R24" t="s">
+        <v>36</v>
+      </c>
+      <c r="S24" t="s">
+        <v>36</v>
+      </c>
+      <c r="T24" t="s">
+        <v>37</v>
+      </c>
+      <c r="U24" t="s">
+        <v>35</v>
+      </c>
+      <c r="V24" t="s">
+        <v>34</v>
+      </c>
+      <c r="W24" t="s">
+        <v>36</v>
+      </c>
+      <c r="X24" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y24" t="s">
+        <v>37</v>
+      </c>
+      <c r="Z24" t="s">
+        <v>34</v>
+      </c>
+      <c r="AA24" t="s">
+        <v>35</v>
+      </c>
+      <c r="AB24" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="25" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A25">
-        <v>31</v>
+        <v>6</v>
       </c>
       <c r="B25">
         <v>111001100013</v>
@@ -2728,10 +2782,10 @@
         <v>28</v>
       </c>
       <c r="D25" t="s">
-        <v>94</v>
+        <v>44</v>
       </c>
       <c r="E25" t="s">
-        <v>95</v>
+        <v>45</v>
       </c>
       <c r="F25" t="s">
         <v>31</v>
@@ -2743,10 +2797,10 @@
         <v>33</v>
       </c>
       <c r="I25" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="J25" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="K25" t="s">
         <v>34</v>
@@ -2758,54 +2812,54 @@
         <v>35</v>
       </c>
       <c r="N25" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="O25" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="P25" t="s">
         <v>35</v>
       </c>
       <c r="Q25" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="R25" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="S25" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="T25" t="s">
         <v>37</v>
       </c>
       <c r="U25" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="V25" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="W25" t="s">
         <v>36</v>
       </c>
       <c r="X25" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Y25" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="Z25" t="s">
         <v>34</v>
       </c>
       <c r="AA25" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="AB25" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="26" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A26">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="B26">
         <v>111001100013</v>
@@ -2814,10 +2868,10 @@
         <v>28</v>
       </c>
       <c r="D26" t="s">
-        <v>44</v>
+        <v>92</v>
       </c>
       <c r="E26" t="s">
-        <v>45</v>
+        <v>93</v>
       </c>
       <c r="F26" t="s">
         <v>31</v>
@@ -2829,13 +2883,13 @@
         <v>33</v>
       </c>
       <c r="I26" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="J26" t="s">
         <v>35</v>
       </c>
       <c r="K26" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="L26" t="s">
         <v>37</v>
@@ -2853,16 +2907,16 @@
         <v>35</v>
       </c>
       <c r="Q26" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="R26" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="S26" t="s">
         <v>35</v>
       </c>
       <c r="T26" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="U26" t="s">
         <v>34</v>
@@ -2871,27 +2925,27 @@
         <v>35</v>
       </c>
       <c r="W26" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="X26" t="s">
         <v>36</v>
       </c>
       <c r="Y26" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="Z26" t="s">
         <v>34</v>
       </c>
       <c r="AA26" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="AB26" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="27" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A27">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B27">
         <v>111001100013</v>
@@ -2900,10 +2954,10 @@
         <v>28</v>
       </c>
       <c r="D27" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="E27" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="F27" t="s">
         <v>31</v>
@@ -2915,13 +2969,13 @@
         <v>33</v>
       </c>
       <c r="I27" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J27" t="s">
         <v>35</v>
       </c>
       <c r="K27" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="L27" t="s">
         <v>37</v>
@@ -2977,7 +3031,7 @@
     </row>
     <row r="28" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A28">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="B28">
         <v>111001100013</v>
@@ -2986,10 +3040,10 @@
         <v>28</v>
       </c>
       <c r="D28" t="s">
-        <v>90</v>
+        <v>52</v>
       </c>
       <c r="E28" t="s">
-        <v>91</v>
+        <v>53</v>
       </c>
       <c r="F28" t="s">
         <v>31</v>
@@ -3025,10 +3079,10 @@
         <v>35</v>
       </c>
       <c r="Q28" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="R28" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="S28" t="s">
         <v>35</v>
@@ -3063,7 +3117,7 @@
     </row>
     <row r="29" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A29">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="B29">
         <v>111001100013</v>
@@ -3072,10 +3126,10 @@
         <v>28</v>
       </c>
       <c r="D29" t="s">
-        <v>52</v>
+        <v>80</v>
       </c>
       <c r="E29" t="s">
-        <v>53</v>
+        <v>81</v>
       </c>
       <c r="F29" t="s">
         <v>31</v>
@@ -3087,7 +3141,7 @@
         <v>33</v>
       </c>
       <c r="I29" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="J29" t="s">
         <v>35</v>
@@ -3105,13 +3159,13 @@
         <v>35</v>
       </c>
       <c r="O29" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="P29" t="s">
         <v>35</v>
       </c>
       <c r="Q29" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="R29" t="s">
         <v>37</v>
@@ -3120,7 +3174,7 @@
         <v>35</v>
       </c>
       <c r="T29" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="U29" t="s">
         <v>34</v>
@@ -3149,7 +3203,7 @@
     </row>
     <row r="30" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A30">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="B30">
         <v>111001100013</v>
@@ -3158,10 +3212,10 @@
         <v>28</v>
       </c>
       <c r="D30" t="s">
-        <v>80</v>
+        <v>64</v>
       </c>
       <c r="E30" t="s">
-        <v>81</v>
+        <v>65</v>
       </c>
       <c r="F30" t="s">
         <v>31</v>
@@ -3173,7 +3227,7 @@
         <v>33</v>
       </c>
       <c r="I30" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="J30" t="s">
         <v>35</v>
@@ -3191,22 +3245,22 @@
         <v>35</v>
       </c>
       <c r="O30" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="P30" t="s">
         <v>35</v>
       </c>
       <c r="Q30" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="R30" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="S30" t="s">
         <v>35</v>
       </c>
       <c r="T30" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="U30" t="s">
         <v>34</v>
@@ -3235,7 +3289,7 @@
     </row>
     <row r="31" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A31">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B31">
         <v>111001100013</v>
@@ -3244,10 +3298,10 @@
         <v>28</v>
       </c>
       <c r="D31" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E31" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="F31" t="s">
         <v>31</v>
@@ -3268,7 +3322,7 @@
         <v>34</v>
       </c>
       <c r="L31" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="M31" t="s">
         <v>35</v>
@@ -3283,10 +3337,10 @@
         <v>35</v>
       </c>
       <c r="Q31" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="R31" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="S31" t="s">
         <v>35</v>
@@ -3321,7 +3375,7 @@
     </row>
     <row r="32" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A32">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="B32">
         <v>111001100013</v>
@@ -3330,10 +3384,10 @@
         <v>28</v>
       </c>
       <c r="D32" t="s">
-        <v>62</v>
+        <v>86</v>
       </c>
       <c r="E32" t="s">
-        <v>63</v>
+        <v>87</v>
       </c>
       <c r="F32" t="s">
         <v>31</v>
@@ -3351,10 +3405,10 @@
         <v>35</v>
       </c>
       <c r="K32" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="L32" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="M32" t="s">
         <v>35</v>
@@ -3369,10 +3423,10 @@
         <v>35</v>
       </c>
       <c r="Q32" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="R32" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S32" t="s">
         <v>35</v>
@@ -3390,7 +3444,7 @@
         <v>34</v>
       </c>
       <c r="X32" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Y32" t="s">
         <v>34</v>
@@ -3407,7 +3461,7 @@
     </row>
     <row r="33" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A33">
-        <v>27</v>
+        <v>59</v>
       </c>
       <c r="B33">
         <v>111001100013</v>
@@ -3416,10 +3470,10 @@
         <v>28</v>
       </c>
       <c r="D33" t="s">
-        <v>86</v>
+        <v>56</v>
       </c>
       <c r="E33" t="s">
-        <v>87</v>
+        <v>57</v>
       </c>
       <c r="F33" t="s">
         <v>31</v>
@@ -3428,72 +3482,72 @@
         <v>32</v>
       </c>
       <c r="H33" t="s">
-        <v>33</v>
+        <v>98</v>
       </c>
       <c r="I33" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="J33" t="s">
         <v>35</v>
       </c>
       <c r="K33" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L33" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="M33" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="N33" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="O33" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="P33" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="Q33" t="s">
         <v>37</v>
       </c>
       <c r="R33" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="S33" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="T33" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="U33" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="V33" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="W33" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="X33" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="Y33" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Z33" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="AA33" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="AB33" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="34" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A34">
-        <v>59</v>
+        <v>34</v>
       </c>
       <c r="B34">
         <v>111001100013</v>
@@ -3502,10 +3556,10 @@
         <v>28</v>
       </c>
       <c r="D34" t="s">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="E34" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="F34" t="s">
         <v>31</v>
@@ -3514,7 +3568,7 @@
         <v>32</v>
       </c>
       <c r="H34" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I34" t="s">
         <v>35</v>
@@ -3523,28 +3577,28 @@
         <v>35</v>
       </c>
       <c r="K34" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="L34" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="M34" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="N34" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="O34" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="P34" t="s">
         <v>34</v>
       </c>
       <c r="Q34" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="R34" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="S34" t="s">
         <v>34</v>
@@ -3553,7 +3607,7 @@
         <v>35</v>
       </c>
       <c r="U34" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="V34" t="s">
         <v>34</v>
@@ -3565,13 +3619,13 @@
         <v>34</v>
       </c>
       <c r="Y34" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Z34" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="AA34" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="AB34" t="s">
         <v>36</v>
@@ -3579,7 +3633,7 @@
     </row>
     <row r="35" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A35">
-        <v>34</v>
+        <v>56</v>
       </c>
       <c r="B35">
         <v>111001100013</v>
@@ -3588,10 +3642,10 @@
         <v>28</v>
       </c>
       <c r="D35" t="s">
-        <v>70</v>
+        <v>58</v>
       </c>
       <c r="E35" t="s">
-        <v>71</v>
+        <v>59</v>
       </c>
       <c r="F35" t="s">
         <v>31</v>
@@ -3600,31 +3654,31 @@
         <v>32</v>
       </c>
       <c r="H35" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I35" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J35" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="K35" t="s">
         <v>37</v>
       </c>
       <c r="L35" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M35" t="s">
         <v>35</v>
       </c>
       <c r="N35" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="O35" t="s">
         <v>34</v>
       </c>
       <c r="P35" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q35" t="s">
         <v>36</v>
@@ -3633,39 +3687,39 @@
         <v>37</v>
       </c>
       <c r="S35" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="T35" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="U35" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="V35" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="W35" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="X35" t="s">
         <v>34</v>
       </c>
       <c r="Y35" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="Z35" t="s">
         <v>35</v>
       </c>
       <c r="AA35" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="AB35" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="36" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A36">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="B36">
         <v>111001100013</v>
@@ -3674,10 +3728,10 @@
         <v>28</v>
       </c>
       <c r="D36" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="E36" t="s">
-        <v>59</v>
+        <v>69</v>
       </c>
       <c r="F36" t="s">
         <v>31</v>
@@ -3686,37 +3740,37 @@
         <v>32</v>
       </c>
       <c r="H36" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I36" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="J36" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="K36" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L36" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="M36" t="s">
         <v>35</v>
       </c>
       <c r="N36" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="O36" t="s">
         <v>34</v>
       </c>
       <c r="P36" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="Q36" t="s">
         <v>36</v>
       </c>
       <c r="R36" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="S36" t="s">
         <v>36</v>
@@ -3725,13 +3779,13 @@
         <v>34</v>
       </c>
       <c r="U36" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="V36" t="s">
         <v>35</v>
       </c>
       <c r="W36" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="X36" t="s">
         <v>34</v>
@@ -3740,18 +3794,18 @@
         <v>34</v>
       </c>
       <c r="Z36" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="AA36" t="s">
         <v>37</v>
       </c>
       <c r="AB36" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="37" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A37">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="B37">
         <v>111001100013</v>
@@ -3760,10 +3814,10 @@
         <v>28</v>
       </c>
       <c r="D37" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
       <c r="E37" t="s">
-        <v>69</v>
+        <v>51</v>
       </c>
       <c r="F37" t="s">
         <v>31</v>
@@ -3772,72 +3826,69 @@
         <v>32</v>
       </c>
       <c r="H37" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I37" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="J37" t="s">
-        <v>34</v>
-      </c>
-      <c r="K37" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="L37" t="s">
         <v>37</v>
       </c>
       <c r="M37" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="N37" t="s">
         <v>34</v>
       </c>
       <c r="O37" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P37" t="s">
         <v>34</v>
       </c>
       <c r="Q37" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="R37" t="s">
         <v>35</v>
       </c>
       <c r="S37" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="T37" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="U37" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="V37" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="W37" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="X37" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="Y37" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Z37" t="s">
         <v>34</v>
       </c>
       <c r="AA37" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="AB37" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="38" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A38">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B38">
         <v>111001100013</v>
@@ -3846,10 +3897,10 @@
         <v>28</v>
       </c>
       <c r="D38" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E38" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F38" t="s">
         <v>31</v>
@@ -3858,69 +3909,72 @@
         <v>32</v>
       </c>
       <c r="H38" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I38" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="J38" t="s">
-        <v>36</v>
+        <v>35</v>
+      </c>
+      <c r="K38" t="s">
+        <v>37</v>
       </c>
       <c r="L38" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="M38" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="N38" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="O38" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="P38" t="s">
         <v>34</v>
       </c>
       <c r="Q38" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="R38" t="s">
         <v>35</v>
       </c>
       <c r="S38" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="T38" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="U38" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="V38" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="W38" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="X38" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Y38" t="s">
         <v>35</v>
       </c>
       <c r="Z38" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="AA38" t="s">
         <v>35</v>
       </c>
       <c r="AB38" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="39" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A39">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="B39">
         <v>111001100013</v>
@@ -3929,10 +3983,10 @@
         <v>28</v>
       </c>
       <c r="D39" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="E39" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="F39" t="s">
         <v>31</v>
@@ -3941,28 +3995,25 @@
         <v>32</v>
       </c>
       <c r="H39" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I39" t="s">
         <v>35</v>
       </c>
       <c r="J39" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="K39" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="L39" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="M39" t="s">
-        <v>35</v>
-      </c>
-      <c r="N39" t="s">
         <v>37</v>
       </c>
       <c r="O39" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="P39" t="s">
         <v>34</v>
@@ -3971,19 +4022,19 @@
         <v>36</v>
       </c>
       <c r="R39" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="S39" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="T39" t="s">
         <v>37</v>
       </c>
       <c r="U39" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="V39" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="W39" t="s">
         <v>34</v>
@@ -3992,21 +4043,21 @@
         <v>35</v>
       </c>
       <c r="Y39" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="Z39" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="AA39" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="AB39" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="40" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A40">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="B40">
         <v>111001100013</v>
@@ -4015,10 +4066,10 @@
         <v>28</v>
       </c>
       <c r="D40" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="E40" t="s">
-        <v>55</v>
+        <v>77</v>
       </c>
       <c r="F40" t="s">
         <v>31</v>
@@ -4027,22 +4078,25 @@
         <v>32</v>
       </c>
       <c r="H40" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I40" t="s">
         <v>35</v>
       </c>
       <c r="J40" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="K40" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="L40" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="M40" t="s">
-        <v>37</v>
+        <v>36</v>
+      </c>
+      <c r="N40" t="s">
+        <v>35</v>
       </c>
       <c r="O40" t="s">
         <v>36</v>
@@ -4054,19 +4108,19 @@
         <v>36</v>
       </c>
       <c r="R40" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="S40" t="s">
         <v>35</v>
       </c>
       <c r="T40" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="U40" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="V40" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="W40" t="s">
         <v>34</v>
@@ -4075,13 +4129,13 @@
         <v>35</v>
       </c>
       <c r="Y40" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Z40" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="AA40" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="AB40" t="s">
         <v>35</v>
@@ -4089,7 +4143,7 @@
     </row>
     <row r="41" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A41">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="B41">
         <v>111001100013</v>
@@ -4098,10 +4152,10 @@
         <v>28</v>
       </c>
       <c r="D41" t="s">
-        <v>76</v>
+        <v>88</v>
       </c>
       <c r="E41" t="s">
-        <v>77</v>
+        <v>89</v>
       </c>
       <c r="F41" t="s">
         <v>31</v>
@@ -4110,25 +4164,25 @@
         <v>32</v>
       </c>
       <c r="H41" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I41" t="s">
         <v>35</v>
       </c>
       <c r="J41" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="K41" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="L41" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="M41" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="N41" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="O41" t="s">
         <v>36</v>
@@ -4140,28 +4194,28 @@
         <v>36</v>
       </c>
       <c r="R41" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="S41" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="T41" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="U41" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="V41" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="W41" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="X41" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="Y41" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Z41" t="s">
         <v>37</v>
@@ -4175,7 +4229,7 @@
     </row>
     <row r="42" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A42">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="B42">
         <v>111001100013</v>
@@ -4184,10 +4238,10 @@
         <v>28</v>
       </c>
       <c r="D42" t="s">
-        <v>88</v>
+        <v>66</v>
       </c>
       <c r="E42" t="s">
-        <v>89</v>
+        <v>67</v>
       </c>
       <c r="F42" t="s">
         <v>31</v>
@@ -4196,19 +4250,19 @@
         <v>32</v>
       </c>
       <c r="H42" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I42" t="s">
         <v>35</v>
       </c>
       <c r="J42" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="K42" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L42" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="M42" t="s">
         <v>35</v>
@@ -4220,13 +4274,13 @@
         <v>36</v>
       </c>
       <c r="P42" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q42" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="R42" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="S42" t="s">
         <v>36</v>
@@ -4235,10 +4289,10 @@
         <v>36</v>
       </c>
       <c r="U42" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="V42" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="W42" t="s">
         <v>35</v>
@@ -4247,13 +4301,13 @@
         <v>34</v>
       </c>
       <c r="Y42" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Z42" t="s">
         <v>37</v>
       </c>
       <c r="AA42" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="AB42" t="s">
         <v>35</v>
@@ -4261,7 +4315,7 @@
     </row>
     <row r="43" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A43">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="B43">
         <v>111001100013</v>
@@ -4270,10 +4324,10 @@
         <v>28</v>
       </c>
       <c r="D43" t="s">
-        <v>66</v>
+        <v>38</v>
       </c>
       <c r="E43" t="s">
-        <v>67</v>
+        <v>39</v>
       </c>
       <c r="F43" t="s">
         <v>31</v>
@@ -4282,28 +4336,28 @@
         <v>32</v>
       </c>
       <c r="H43" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I43" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="J43" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="K43" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="L43" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="M43" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="N43" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="O43" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="P43" t="s">
         <v>35</v>
@@ -4315,39 +4369,39 @@
         <v>37</v>
       </c>
       <c r="S43" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="T43" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="U43" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="V43" t="s">
         <v>34</v>
       </c>
       <c r="W43" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="X43" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Y43" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="Z43" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="AA43" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="AB43" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="44" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A44">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="B44">
         <v>111001100013</v>
@@ -4356,10 +4410,10 @@
         <v>28</v>
       </c>
       <c r="D44" t="s">
-        <v>38</v>
+        <v>96</v>
       </c>
       <c r="E44" t="s">
-        <v>39</v>
+        <v>97</v>
       </c>
       <c r="F44" t="s">
         <v>31</v>
@@ -4368,10 +4422,10 @@
         <v>32</v>
       </c>
       <c r="H44" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I44" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="J44" t="s">
         <v>34</v>
@@ -4383,46 +4437,46 @@
         <v>36</v>
       </c>
       <c r="M44" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="N44" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="O44" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P44" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q44" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="R44" t="s">
         <v>37</v>
       </c>
       <c r="S44" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="T44" t="s">
         <v>34</v>
       </c>
       <c r="U44" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="V44" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="W44" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="X44" t="s">
         <v>35</v>
       </c>
       <c r="Y44" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="Z44" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="AA44" t="s">
         <v>34</v>
@@ -4433,7 +4487,7 @@
     </row>
     <row r="45" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A45">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B45">
         <v>111001100013</v>
@@ -4442,10 +4496,10 @@
         <v>28</v>
       </c>
       <c r="D45" t="s">
-        <v>96</v>
+        <v>60</v>
       </c>
       <c r="E45" t="s">
-        <v>97</v>
+        <v>61</v>
       </c>
       <c r="F45" t="s">
         <v>31</v>
@@ -4454,7 +4508,7 @@
         <v>32</v>
       </c>
       <c r="H45" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I45" t="s">
         <v>35</v>
@@ -4466,60 +4520,60 @@
         <v>37</v>
       </c>
       <c r="L45" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="M45" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="N45" t="s">
         <v>37</v>
       </c>
       <c r="O45" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P45" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="Q45" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="R45" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="S45" t="s">
         <v>37</v>
       </c>
       <c r="T45" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="U45" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="V45" t="s">
         <v>35</v>
       </c>
       <c r="W45" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="X45" t="s">
         <v>35</v>
       </c>
       <c r="Y45" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="Z45" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="AA45" t="s">
         <v>34</v>
       </c>
       <c r="AB45" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="46" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A46">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B46">
         <v>111001100013</v>
@@ -4528,10 +4582,10 @@
         <v>28</v>
       </c>
       <c r="D46" t="s">
-        <v>60</v>
+        <v>78</v>
       </c>
       <c r="E46" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="F46" t="s">
         <v>31</v>
@@ -4540,7 +4594,7 @@
         <v>32</v>
       </c>
       <c r="H46" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I46" t="s">
         <v>35</v>
@@ -4573,13 +4627,13 @@
         <v>34</v>
       </c>
       <c r="S46" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="T46" t="s">
         <v>36</v>
       </c>
       <c r="U46" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="V46" t="s">
         <v>35</v>
@@ -4588,24 +4642,24 @@
         <v>34</v>
       </c>
       <c r="X46" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="Y46" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="Z46" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="AA46" t="s">
         <v>34</v>
       </c>
       <c r="AB46" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="47" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A47">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B47">
         <v>111001100013</v>
@@ -4614,10 +4668,10 @@
         <v>28</v>
       </c>
       <c r="D47" t="s">
-        <v>78</v>
+        <v>40</v>
       </c>
       <c r="E47" t="s">
-        <v>79</v>
+        <v>41</v>
       </c>
       <c r="F47" t="s">
         <v>31</v>
@@ -4626,7 +4680,7 @@
         <v>32</v>
       </c>
       <c r="H47" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I47" t="s">
         <v>35</v>
@@ -4641,28 +4695,28 @@
         <v>35</v>
       </c>
       <c r="M47" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="N47" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="O47" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="P47" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="Q47" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="R47" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S47" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="T47" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="U47" t="s">
         <v>37</v>
@@ -4671,27 +4725,27 @@
         <v>35</v>
       </c>
       <c r="W47" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="X47" t="s">
         <v>34</v>
       </c>
       <c r="Y47" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Z47" t="s">
         <v>37</v>
       </c>
       <c r="AA47" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="AB47" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="48" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A48">
-        <v>39</v>
+        <v>58</v>
       </c>
       <c r="B48">
         <v>111001100013</v>
@@ -4700,10 +4754,10 @@
         <v>28</v>
       </c>
       <c r="D48" t="s">
-        <v>40</v>
+        <v>72</v>
       </c>
       <c r="E48" t="s">
-        <v>41</v>
+        <v>73</v>
       </c>
       <c r="F48" t="s">
         <v>31</v>
@@ -4712,7 +4766,7 @@
         <v>32</v>
       </c>
       <c r="H48" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I48" t="s">
         <v>35</v>
@@ -4721,40 +4775,40 @@
         <v>34</v>
       </c>
       <c r="K48" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L48" t="s">
         <v>35</v>
       </c>
       <c r="M48" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="N48" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="O48" t="s">
         <v>34</v>
       </c>
       <c r="P48" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="Q48" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="R48" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="S48" t="s">
         <v>35</v>
       </c>
       <c r="T48" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="U48" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="V48" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="W48" t="s">
         <v>35</v>
@@ -4766,18 +4820,18 @@
         <v>37</v>
       </c>
       <c r="Z48" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="AA48" t="s">
         <v>36</v>
       </c>
       <c r="AB48" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="49" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A49">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B49">
         <v>111001100013</v>
@@ -4786,10 +4840,10 @@
         <v>28</v>
       </c>
       <c r="D49" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E49" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F49" t="s">
         <v>31</v>
@@ -4798,19 +4852,19 @@
         <v>32</v>
       </c>
       <c r="H49" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I49" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="J49" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="K49" t="s">
         <v>34</v>
       </c>
       <c r="L49" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="M49" t="s">
         <v>35</v>
@@ -4819,10 +4873,10 @@
         <v>37</v>
       </c>
       <c r="O49" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="P49" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="Q49" t="s">
         <v>36</v>
@@ -4831,7 +4885,7 @@
         <v>37</v>
       </c>
       <c r="S49" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="T49" t="s">
         <v>35</v>
@@ -4840,7 +4894,7 @@
         <v>34</v>
       </c>
       <c r="V49" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="W49" t="s">
         <v>35</v>
@@ -4849,21 +4903,21 @@
         <v>34</v>
       </c>
       <c r="Y49" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Z49" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="AA49" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="AB49" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="50" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A50">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="B50">
         <v>111001100013</v>
@@ -4872,10 +4926,10 @@
         <v>28</v>
       </c>
       <c r="D50" t="s">
-        <v>74</v>
+        <v>46</v>
       </c>
       <c r="E50" t="s">
-        <v>75</v>
+        <v>47</v>
       </c>
       <c r="F50" t="s">
         <v>31</v>
@@ -4884,31 +4938,31 @@
         <v>32</v>
       </c>
       <c r="H50" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I50" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="J50" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="K50" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="L50" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="M50" t="s">
         <v>35</v>
       </c>
       <c r="N50" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="O50" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="P50" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="Q50" t="s">
         <v>36</v>
@@ -4917,39 +4971,39 @@
         <v>37</v>
       </c>
       <c r="S50" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="T50" t="s">
         <v>35</v>
       </c>
       <c r="U50" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="V50" t="s">
         <v>35</v>
       </c>
       <c r="W50" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="X50" t="s">
         <v>34</v>
       </c>
       <c r="Y50" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="Z50" t="s">
         <v>37</v>
       </c>
       <c r="AA50" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="AB50" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="51" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A51">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="B51">
         <v>111001100013</v>
@@ -4958,10 +5012,10 @@
         <v>28</v>
       </c>
       <c r="D51" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="E51" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="F51" t="s">
         <v>31</v>
@@ -4970,72 +5024,72 @@
         <v>32</v>
       </c>
       <c r="H51" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I51" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J51" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="K51" t="s">
         <v>37</v>
       </c>
       <c r="L51" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M51" t="s">
         <v>35</v>
       </c>
       <c r="N51" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="O51" t="s">
         <v>34</v>
       </c>
       <c r="P51" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="Q51" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="R51" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="S51" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="T51" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="U51" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="V51" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="W51" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="X51" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Y51" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="Z51" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="AA51" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="AB51" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="52" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A52">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B52">
         <v>111001100013</v>
@@ -5044,10 +5098,10 @@
         <v>28</v>
       </c>
       <c r="D52" t="s">
-        <v>42</v>
+        <v>82</v>
       </c>
       <c r="E52" t="s">
-        <v>43</v>
+        <v>83</v>
       </c>
       <c r="F52" t="s">
         <v>31</v>
@@ -5056,58 +5110,58 @@
         <v>32</v>
       </c>
       <c r="H52" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I52" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="J52" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="K52" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L52" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="M52" t="s">
         <v>35</v>
       </c>
       <c r="N52" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="O52" t="s">
         <v>34</v>
       </c>
       <c r="P52" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="Q52" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="R52" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="S52" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="T52" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="U52" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="V52" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="W52" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="X52" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="Y52" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Z52" t="s">
         <v>35</v>
@@ -5116,12 +5170,12 @@
         <v>36</v>
       </c>
       <c r="AB52" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="53" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A53">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="B53">
         <v>111001100013</v>
@@ -5130,10 +5184,10 @@
         <v>28</v>
       </c>
       <c r="D53" t="s">
-        <v>82</v>
+        <v>29</v>
       </c>
       <c r="E53" t="s">
-        <v>83</v>
+        <v>30</v>
       </c>
       <c r="F53" t="s">
         <v>31</v>
@@ -5142,7 +5196,7 @@
         <v>32</v>
       </c>
       <c r="H53" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I53" t="s">
         <v>35</v>
@@ -5154,13 +5208,13 @@
         <v>34</v>
       </c>
       <c r="L53" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="M53" t="s">
         <v>35</v>
       </c>
       <c r="N53" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="O53" t="s">
         <v>34</v>
@@ -5175,7 +5229,7 @@
         <v>35</v>
       </c>
       <c r="S53" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="T53" t="s">
         <v>34</v>
@@ -5187,27 +5241,27 @@
         <v>35</v>
       </c>
       <c r="W53" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="X53" t="s">
         <v>34</v>
       </c>
       <c r="Y53" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="Z53" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="AA53" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="AB53" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="54" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A54">
-        <v>37</v>
+        <v>51</v>
       </c>
       <c r="B54">
         <v>111001100013</v>
@@ -5216,10 +5270,10 @@
         <v>28</v>
       </c>
       <c r="D54" t="s">
-        <v>29</v>
+        <v>84</v>
       </c>
       <c r="E54" t="s">
-        <v>30</v>
+        <v>85</v>
       </c>
       <c r="F54" t="s">
         <v>31</v>
@@ -5228,19 +5282,19 @@
         <v>32</v>
       </c>
       <c r="H54" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I54" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J54" t="s">
         <v>34</v>
       </c>
       <c r="K54" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="L54" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="M54" t="s">
         <v>35</v>
@@ -5249,51 +5303,51 @@
         <v>37</v>
       </c>
       <c r="O54" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P54" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="Q54" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="R54" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="S54" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="T54" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="U54" t="s">
         <v>36</v>
       </c>
       <c r="V54" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="W54" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="X54" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Y54" t="s">
         <v>34</v>
       </c>
       <c r="Z54" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="AA54" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="AB54" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="55" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A55">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="B55">
         <v>111001100013</v>
@@ -5302,10 +5356,10 @@
         <v>28</v>
       </c>
       <c r="D55" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="E55" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="F55" t="s">
         <v>31</v>
@@ -5314,13 +5368,13 @@
         <v>32</v>
       </c>
       <c r="H55" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I55" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J55" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="K55" t="s">
         <v>37</v>
@@ -5332,7 +5386,7 @@
         <v>35</v>
       </c>
       <c r="N55" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="O55" t="s">
         <v>35</v>
@@ -5341,71 +5395,131 @@
         <v>35</v>
       </c>
       <c r="Q55" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="R55" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="S55" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="T55" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="U55" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="V55" t="s">
         <v>34</v>
       </c>
       <c r="W55" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="X55" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="Y55" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="Z55" t="s">
         <v>35</v>
       </c>
       <c r="AA55" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="AB55" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="56" spans="1:28" x14ac:dyDescent="0.35">
-      <c r="A56">
-        <v>65</v>
+      <c r="A56" s="2">
+        <v>36</v>
       </c>
       <c r="B56">
         <v>111001100013</v>
       </c>
-      <c r="C56" t="s">
-        <v>28</v>
-      </c>
-      <c r="D56" t="s">
+      <c r="C56" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E56" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F56" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H56" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="E56" t="s">
-        <v>99</v>
-      </c>
-      <c r="F56" t="s">
-        <v>31</v>
-      </c>
-      <c r="G56" t="s">
-        <v>32</v>
-      </c>
-      <c r="H56" t="s">
-        <v>100</v>
+      <c r="I56" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="J56" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="K56" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="L56" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="M56" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="N56" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="O56" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="P56" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q56" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="R56" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="S56" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="T56" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="U56" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="V56" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="W56" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="X56" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y56" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Z56" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="AA56" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="AB56" s="2" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="57" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A57">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="B57">
         <v>111001100013</v>
@@ -5414,10 +5528,10 @@
         <v>28</v>
       </c>
       <c r="D57" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E57" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="F57" t="s">
         <v>31</v>
@@ -5426,22 +5540,22 @@
         <v>32</v>
       </c>
       <c r="H57" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I57" t="s">
         <v>35</v>
       </c>
       <c r="J57" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="K57" t="s">
         <v>37</v>
       </c>
       <c r="L57" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M57" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="N57" t="s">
         <v>36</v>
@@ -5450,134 +5564,134 @@
         <v>35</v>
       </c>
       <c r="P57" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q57" t="s">
         <v>37</v>
       </c>
       <c r="R57" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S57" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="T57" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="U57" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="V57" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="W57" t="s">
         <v>35</v>
       </c>
       <c r="X57" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="Y57" t="s">
         <v>36</v>
       </c>
       <c r="Z57" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="AA57" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="AB57" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="58" spans="1:28" x14ac:dyDescent="0.35">
-      <c r="A58" s="2">
-        <v>36</v>
+      <c r="A58">
+        <v>46</v>
       </c>
       <c r="B58">
         <v>111001100013</v>
       </c>
-      <c r="C58" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D58" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="E58" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="F58" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="G58" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="H58" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="I58" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="J58" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="K58" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="L58" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="M58" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="N58" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="O58" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="P58" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="Q58" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="R58" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="S58" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="T58" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="U58" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="V58" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="W58" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="X58" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y58" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="Z58" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="AA58" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="AB58" s="2" t="s">
-        <v>34</v>
+      <c r="C58" t="s">
+        <v>28</v>
+      </c>
+      <c r="D58" t="s">
+        <v>90</v>
+      </c>
+      <c r="E58" t="s">
+        <v>91</v>
+      </c>
+      <c r="F58" t="s">
+        <v>31</v>
+      </c>
+      <c r="G58" t="s">
+        <v>32</v>
+      </c>
+      <c r="H58" t="s">
+        <v>98</v>
+      </c>
+      <c r="I58" t="s">
+        <v>35</v>
+      </c>
+      <c r="J58" t="s">
+        <v>34</v>
+      </c>
+      <c r="K58" t="s">
+        <v>37</v>
+      </c>
+      <c r="L58" t="s">
+        <v>35</v>
+      </c>
+      <c r="M58" t="s">
+        <v>35</v>
+      </c>
+      <c r="N58" t="s">
+        <v>36</v>
+      </c>
+      <c r="O58" t="s">
+        <v>34</v>
+      </c>
+      <c r="P58" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q58" t="s">
+        <v>36</v>
+      </c>
+      <c r="R58" t="s">
+        <v>35</v>
+      </c>
+      <c r="S58" t="s">
+        <v>34</v>
+      </c>
+      <c r="T58" t="s">
+        <v>35</v>
+      </c>
+      <c r="U58" t="s">
+        <v>37</v>
+      </c>
+      <c r="V58" t="s">
+        <v>35</v>
+      </c>
+      <c r="W58" t="s">
+        <v>35</v>
+      </c>
+      <c r="X58" t="s">
+        <v>34</v>
+      </c>
+      <c r="Y58" t="s">
+        <v>34</v>
+      </c>
+      <c r="Z58" t="s">
+        <v>36</v>
+      </c>
+      <c r="AA58" t="s">
+        <v>35</v>
+      </c>
+      <c r="AB58" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="59" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A59">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="B59">
         <v>111001100013</v>
@@ -5586,10 +5700,10 @@
         <v>28</v>
       </c>
       <c r="D59" t="s">
-        <v>92</v>
+        <v>52</v>
       </c>
       <c r="E59" t="s">
-        <v>93</v>
+        <v>53</v>
       </c>
       <c r="F59" t="s">
         <v>31</v>
@@ -5598,64 +5712,64 @@
         <v>32</v>
       </c>
       <c r="H59" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I59" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="J59" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="K59" t="s">
         <v>37</v>
       </c>
       <c r="L59" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="M59" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="N59" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="O59" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="P59" t="s">
         <v>36</v>
       </c>
       <c r="Q59" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="R59" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="S59" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="T59" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="U59" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="V59" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="W59" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="X59" t="s">
         <v>34</v>
       </c>
       <c r="Y59" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Z59" t="s">
         <v>36</v>
       </c>
       <c r="AA59" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="AB59" t="s">
         <v>37</v>
@@ -5663,7 +5777,7 @@
     </row>
     <row r="60" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A60">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="B60">
         <v>111001100013</v>
@@ -5672,10 +5786,10 @@
         <v>28</v>
       </c>
       <c r="D60" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="E60" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="F60" t="s">
         <v>31</v>
@@ -5684,7 +5798,7 @@
         <v>32</v>
       </c>
       <c r="H60" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I60" t="s">
         <v>35</v>
@@ -5692,9 +5806,6 @@
       <c r="J60" t="s">
         <v>34</v>
       </c>
-      <c r="K60" t="s">
-        <v>37</v>
-      </c>
       <c r="L60" t="s">
         <v>35</v>
       </c>
@@ -5702,7 +5813,7 @@
         <v>35</v>
       </c>
       <c r="N60" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="O60" t="s">
         <v>34</v>
@@ -5714,19 +5825,19 @@
         <v>36</v>
       </c>
       <c r="R60" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="S60" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="T60" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="U60" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="V60" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="W60" t="s">
         <v>35</v>
@@ -5735,13 +5846,13 @@
         <v>34</v>
       </c>
       <c r="Y60" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="Z60" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="AA60" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="AB60" t="s">
         <v>35</v>
@@ -5749,7 +5860,7 @@
     </row>
     <row r="61" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A61">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B61">
         <v>111001100013</v>
@@ -5758,10 +5869,10 @@
         <v>28</v>
       </c>
       <c r="D61" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="E61" t="s">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="F61" t="s">
         <v>31</v>
@@ -5770,7 +5881,7 @@
         <v>32</v>
       </c>
       <c r="H61" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I61" t="s">
         <v>37</v>
@@ -5806,7 +5917,7 @@
         <v>37</v>
       </c>
       <c r="T61" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="U61" t="s">
         <v>34</v>
@@ -5824,7 +5935,7 @@
         <v>37</v>
       </c>
       <c r="Z61" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="AA61" t="s">
         <v>35</v>
@@ -5835,7 +5946,7 @@
     </row>
     <row r="62" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A62">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="B62">
         <v>111001100013</v>
@@ -5844,10 +5955,10 @@
         <v>28</v>
       </c>
       <c r="D62" t="s">
-        <v>80</v>
+        <v>62</v>
       </c>
       <c r="E62" t="s">
-        <v>81</v>
+        <v>63</v>
       </c>
       <c r="F62" t="s">
         <v>31</v>
@@ -5856,28 +5967,31 @@
         <v>32</v>
       </c>
       <c r="H62" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I62" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="J62" t="s">
         <v>34</v>
       </c>
+      <c r="K62" t="s">
+        <v>37</v>
+      </c>
       <c r="L62" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="M62" t="s">
         <v>35</v>
       </c>
       <c r="N62" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="O62" t="s">
         <v>34</v>
       </c>
       <c r="P62" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="Q62" t="s">
         <v>36</v>
@@ -5886,16 +6000,16 @@
         <v>37</v>
       </c>
       <c r="S62" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="T62" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="U62" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="V62" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="W62" t="s">
         <v>35</v>
@@ -5904,13 +6018,13 @@
         <v>34</v>
       </c>
       <c r="Y62" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="Z62" t="s">
         <v>37</v>
       </c>
       <c r="AA62" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="AB62" t="s">
         <v>35</v>
@@ -5918,7 +6032,7 @@
     </row>
     <row r="63" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A63">
-        <v>62</v>
+        <v>49</v>
       </c>
       <c r="B63">
         <v>111001100013</v>
@@ -5927,10 +6041,10 @@
         <v>28</v>
       </c>
       <c r="D63" t="s">
-        <v>64</v>
+        <v>86</v>
       </c>
       <c r="E63" t="s">
-        <v>65</v>
+        <v>87</v>
       </c>
       <c r="F63" t="s">
         <v>31</v>
@@ -5939,247 +6053,76 @@
         <v>32</v>
       </c>
       <c r="H63" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I63" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="J63" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="K63" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L63" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="M63" t="s">
         <v>35</v>
       </c>
       <c r="N63" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="O63" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P63" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="Q63" t="s">
         <v>36</v>
       </c>
       <c r="R63" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="S63" t="s">
         <v>37</v>
       </c>
       <c r="T63" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="U63" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="V63" t="s">
         <v>34</v>
       </c>
       <c r="W63" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="X63" t="s">
         <v>34</v>
       </c>
       <c r="Y63" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="Z63" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="AA63" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="AB63" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="64" spans="1:28" x14ac:dyDescent="0.35">
-      <c r="A64">
-        <v>64</v>
-      </c>
-      <c r="B64">
-        <v>111001100013</v>
-      </c>
-      <c r="C64" t="s">
-        <v>28</v>
-      </c>
-      <c r="D64" t="s">
-        <v>62</v>
-      </c>
-      <c r="E64" t="s">
-        <v>63</v>
-      </c>
-      <c r="F64" t="s">
-        <v>31</v>
-      </c>
-      <c r="G64" t="s">
-        <v>32</v>
-      </c>
-      <c r="H64" t="s">
-        <v>100</v>
-      </c>
-      <c r="I64" t="s">
-        <v>37</v>
-      </c>
-      <c r="J64" t="s">
-        <v>34</v>
-      </c>
-      <c r="K64" t="s">
-        <v>37</v>
-      </c>
-      <c r="L64" t="s">
-        <v>37</v>
-      </c>
-      <c r="M64" t="s">
-        <v>35</v>
-      </c>
-      <c r="N64" t="s">
-        <v>34</v>
-      </c>
-      <c r="O64" t="s">
-        <v>34</v>
-      </c>
-      <c r="P64" t="s">
-        <v>35</v>
-      </c>
-      <c r="Q64" t="s">
-        <v>36</v>
-      </c>
-      <c r="R64" t="s">
-        <v>37</v>
-      </c>
-      <c r="S64" t="s">
-        <v>36</v>
-      </c>
-      <c r="T64" t="s">
-        <v>34</v>
-      </c>
-      <c r="U64" t="s">
-        <v>35</v>
-      </c>
-      <c r="V64" t="s">
-        <v>35</v>
-      </c>
-      <c r="W64" t="s">
-        <v>35</v>
-      </c>
-      <c r="X64" t="s">
-        <v>34</v>
-      </c>
-      <c r="Y64" t="s">
-        <v>34</v>
-      </c>
-      <c r="Z64" t="s">
-        <v>37</v>
-      </c>
-      <c r="AA64" t="s">
-        <v>37</v>
-      </c>
-      <c r="AB64" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="65" spans="1:28" x14ac:dyDescent="0.35">
-      <c r="A65">
-        <v>49</v>
-      </c>
-      <c r="B65">
-        <v>111001100013</v>
-      </c>
-      <c r="C65" t="s">
-        <v>28</v>
-      </c>
-      <c r="D65" t="s">
-        <v>86</v>
-      </c>
-      <c r="E65" t="s">
-        <v>87</v>
-      </c>
-      <c r="F65" t="s">
-        <v>31</v>
-      </c>
-      <c r="G65" t="s">
-        <v>32</v>
-      </c>
-      <c r="H65" t="s">
-        <v>100</v>
-      </c>
-      <c r="I65" t="s">
-        <v>35</v>
-      </c>
-      <c r="J65" t="s">
-        <v>35</v>
-      </c>
-      <c r="K65" t="s">
-        <v>34</v>
-      </c>
-      <c r="L65" t="s">
-        <v>37</v>
-      </c>
-      <c r="M65" t="s">
-        <v>35</v>
-      </c>
-      <c r="N65" t="s">
-        <v>37</v>
-      </c>
-      <c r="O65" t="s">
-        <v>35</v>
-      </c>
-      <c r="P65" t="s">
-        <v>34</v>
-      </c>
-      <c r="Q65" t="s">
-        <v>36</v>
-      </c>
-      <c r="R65" t="s">
-        <v>37</v>
-      </c>
-      <c r="S65" t="s">
-        <v>37</v>
-      </c>
-      <c r="T65" t="s">
-        <v>34</v>
-      </c>
-      <c r="U65" t="s">
-        <v>37</v>
-      </c>
-      <c r="V65" t="s">
-        <v>34</v>
-      </c>
-      <c r="W65" t="s">
-        <v>35</v>
-      </c>
-      <c r="X65" t="s">
-        <v>34</v>
-      </c>
-      <c r="Y65" t="s">
-        <v>34</v>
-      </c>
-      <c r="Z65" t="s">
-        <v>37</v>
-      </c>
-      <c r="AA65" t="s">
-        <v>36</v>
-      </c>
-      <c r="AB65" t="s">
         <v>36</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="E1:E33">
-    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
+  <autoFilter ref="A1:AB63" xr:uid="{ADB2070B-47CF-4426-A87A-6271E231ACA6}"/>
+  <conditionalFormatting sqref="E33:E63">
+    <cfRule type="duplicateValues" dxfId="1" priority="3"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E34:E65">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  <conditionalFormatting sqref="E1:E32">
+    <cfRule type="duplicateValues" dxfId="0" priority="4"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>